<commit_message>
Adding ExcelUtil, ContactExcelData and MailExcelData to Github repository
</commit_message>
<xml_diff>
--- a/ExcelData/Excel Data.xlsx
+++ b/ExcelData/Excel Data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Appium\CI_CD_Jenkins_Git_Github\ExcelData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Appium\Framework_Krishna3750\ExcelData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA2C75BF-F88E-4CE1-B973-3980F0AEB571}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7D97192-8CAA-4025-82CC-574A75D26958}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{8F3CF768-72B3-4C85-BE69-CD56609A6B15}"/>
+    <workbookView xWindow="3564" yWindow="1704" windowWidth="15624" windowHeight="8964" xr2:uid="{8F3CF768-72B3-4C85-BE69-CD56609A6B15}"/>
   </bookViews>
   <sheets>
     <sheet name="Phone" sheetId="1" r:id="rId1"/>
@@ -170,17 +170,17 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="14"/>
-      <color theme="1"/>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
+      <b/>
+      <sz val="13"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -205,18 +205,18 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -543,210 +543,211 @@
     <col min="6" max="6" width="19.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="18" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:6" ht="17.399999999999999" x14ac:dyDescent="0.35">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="4" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="2"/>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
+      <c r="A2" s="1"/>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2" t="s">
+      <c r="B3" s="1"/>
+      <c r="C3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="F3" s="2">
+      <c r="F3" s="1">
         <v>6907123987</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2" t="s">
+      <c r="B4" s="1"/>
+      <c r="C4" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="F4" s="2">
+      <c r="F4" s="1">
         <v>7091430912</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="2"/>
-      <c r="C5" s="2" t="s">
+      <c r="B5" s="1"/>
+      <c r="C5" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="E5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="F5" s="2">
+      <c r="F5" s="1">
         <v>9124560912</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="2"/>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
+      <c r="A6" s="1"/>
+      <c r="B6" s="1"/>
+      <c r="C6" s="1"/>
+      <c r="D6" s="1"/>
+      <c r="E6" s="1"/>
+      <c r="F6" s="1"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="D7" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="E7" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F7" s="2">
+      <c r="F7" s="1">
         <v>7891230764</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="D8" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="E8" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F8" s="2">
+      <c r="F8" s="1">
         <v>9105680912</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" s="2" t="s">
+      <c r="A9" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C9" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="D9" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="E9" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="F9" s="2">
+      <c r="F9" s="1">
         <v>6091526792</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A10" s="2"/>
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
+      <c r="A10" s="1"/>
+      <c r="B10" s="1"/>
+      <c r="C10" s="1"/>
+      <c r="D10" s="1"/>
+      <c r="E10" s="1"/>
+      <c r="F10" s="1"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A11" s="2" t="s">
+      <c r="A11" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
+      <c r="C11" s="1"/>
+      <c r="D11" s="1"/>
+      <c r="E11" s="1"/>
+      <c r="F11" s="1"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A12" s="2" t="s">
+      <c r="A12" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
+      <c r="C12" s="1"/>
+      <c r="D12" s="1"/>
+      <c r="E12" s="1"/>
+      <c r="F12" s="1"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A13" s="2" t="s">
+      <c r="A13" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-      <c r="F13" s="2"/>
+      <c r="C13" s="1"/>
+      <c r="D13" s="1"/>
+      <c r="E13" s="1"/>
+      <c r="F13" s="1"/>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A14" s="2"/>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
+      <c r="A14" s="1"/>
+      <c r="B14" s="1"/>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
+      <c r="E14" s="1"/>
+      <c r="F14" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -761,7 +762,7 @@
     <col min="6" max="6" width="12.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="18" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" ht="17.399999999999999" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -779,7 +780,7 @@
       <c r="A3" t="s">
         <v>32</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="2" t="s">
         <v>33</v>
       </c>
       <c r="C3" t="s">
@@ -790,7 +791,7 @@
       <c r="A4" t="s">
         <v>32</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="2" t="s">
         <v>35</v>
       </c>
       <c r="C4" t="s">
@@ -801,7 +802,7 @@
       <c r="A5" t="s">
         <v>32</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="2" t="s">
         <v>37</v>
       </c>
       <c r="C5" t="s">
@@ -812,7 +813,7 @@
       <c r="A7" t="s">
         <v>39</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="2" t="s">
         <v>33</v>
       </c>
       <c r="D7" t="s">
@@ -823,7 +824,7 @@
       <c r="A8" t="s">
         <v>39</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="2" t="s">
         <v>35</v>
       </c>
       <c r="D8" t="s">
@@ -834,7 +835,7 @@
       <c r="A9" t="s">
         <v>39</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="2" t="s">
         <v>37</v>
       </c>
       <c r="D9" t="s">
@@ -851,5 +852,6 @@
     <hyperlink ref="B9" r:id="rId6" xr:uid="{47AF4D32-FDC3-43E7-9974-11D8BD48E1B7}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId7"/>
 </worksheet>
 </file>
</xml_diff>